<commit_message>
ajout des vto dans leur liste
</commit_message>
<xml_diff>
--- a/Liste VTO.xlsx
+++ b/Liste VTO.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dossier LOUMA\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_62E75E214BEF08387827ABE3F4F2BDEBE23AB00D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDCB5D04-E430-4269-A0E8-20CA2EEAA14D}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste VTO" sheetId="1" r:id="rId1"/>
@@ -17,17 +18,28 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste VTO'!$A$1:$F$45</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="160">
   <si>
     <t>DRV</t>
   </si>
@@ -149,6 +161,9 @@
     <t>pvt_dfallf0271</t>
   </si>
   <si>
+    <t> 787657059</t>
+  </si>
+  <si>
     <t xml:space="preserve">NDEYE </t>
   </si>
   <si>
@@ -470,14 +485,47 @@
     <t>pvt_tbogo1719</t>
   </si>
   <si>
-    <t> 787657059</t>
+    <t>IBRAHIMA SENE(SADI ZPPG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KHADIM </t>
+  </si>
+  <si>
+    <t>NIANG</t>
+  </si>
+  <si>
+    <t>Pvt_ibsen0464</t>
+  </si>
+  <si>
+    <t>CHEIKH</t>
+  </si>
+  <si>
+    <t>Pvt_ibsen0440</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOUSSO </t>
+  </si>
+  <si>
+    <t>BADIANE</t>
+  </si>
+  <si>
+    <t>Pvt_ibsen0253</t>
+  </si>
+  <si>
+    <t>MAIMOUNA</t>
+  </si>
+  <si>
+    <t>CAMARA</t>
+  </si>
+  <si>
+    <t>Pvt_ibsen0239</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -499,6 +547,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -514,7 +568,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -574,11 +628,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -588,6 +670,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -605,6 +693,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -885,18 +982,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="58.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" customWidth="1"/>
+    <col min="2" max="2" width="58.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -916,11 +1013,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -936,9 +1033,9 @@
         <v>782989910</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="6"/>
-      <c r="B3" s="9"/>
+    <row r="3" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A3" s="8"/>
+      <c r="B3" s="11"/>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
@@ -952,9 +1049,9 @@
         <v>787095594</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="6"/>
-      <c r="B4" s="9"/>
+    <row r="4" spans="1:6">
+      <c r="A4" s="8"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
@@ -968,9 +1065,9 @@
         <v>781180981</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="7"/>
-      <c r="B5" s="10"/>
+    <row r="5" spans="1:6">
+      <c r="A5" s="9"/>
+      <c r="B5" s="12"/>
       <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
@@ -984,11 +1081,11 @@
         <v>787095584</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:6">
+      <c r="A6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -1004,9 +1101,9 @@
         <v>786241266</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="6"/>
-      <c r="B7" s="9" t="s">
+    <row r="7" spans="1:6" ht="14.45">
+      <c r="A7" s="8"/>
+      <c r="B7" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1022,9 +1119,9 @@
         <v>789160174</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="6"/>
-      <c r="B8" s="9" t="s">
+    <row r="8" spans="1:6" ht="14.45">
+      <c r="A8" s="8"/>
+      <c r="B8" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -1040,9 +1137,9 @@
         <v>786241255</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="7"/>
-      <c r="B9" s="10" t="s">
+    <row r="9" spans="1:6" ht="14.45">
+      <c r="A9" s="9"/>
+      <c r="B9" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -1058,11 +1155,11 @@
         <v>775812208</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:6" ht="14.45">
+      <c r="A10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="10" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1078,9 +1175,9 @@
         <v>789166714</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="1:6" ht="14.45">
+      <c r="A11" s="8"/>
+      <c r="B11" s="11" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1093,667 +1190,748 @@
         <v>39</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="6"/>
-      <c r="B12" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="14.45">
+      <c r="A12" s="8"/>
+      <c r="B12" s="11" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2">
         <v>789166702</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="7"/>
-      <c r="B13" s="10" t="s">
+    <row r="13" spans="1:6" ht="14.45">
+      <c r="A13" s="9"/>
+      <c r="B13" s="12" t="s">
         <v>33</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F13" s="2">
         <v>787655205</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="8" t="s">
+    <row r="14" spans="1:6" ht="14.45">
+      <c r="A14" s="7" t="s">
         <v>46</v>
       </c>
+      <c r="B14" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="C14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="14.45">
+      <c r="A15" s="8"/>
+      <c r="B15" s="11" t="s">
         <v>47</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="6"/>
-      <c r="B15" s="9" t="s">
-        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F15" s="2">
         <v>787080726</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="6"/>
-      <c r="B16" s="9" t="s">
-        <v>46</v>
+    <row r="16" spans="1:6" ht="14.45">
+      <c r="A16" s="8"/>
+      <c r="B16" s="11" t="s">
+        <v>47</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F16" s="2">
         <v>787081068</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="7"/>
-      <c r="B17" s="10" t="s">
-        <v>46</v>
+    <row r="17" spans="1:6" ht="14.45">
+      <c r="A17" s="9"/>
+      <c r="B17" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F17" s="2">
         <v>781590999</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" s="8" t="s">
+    <row r="18" spans="1:6" ht="14.45">
+      <c r="A18" s="7" t="s">
         <v>59</v>
       </c>
+      <c r="B18" s="10" t="s">
+        <v>60</v>
+      </c>
       <c r="C18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="14.45">
+      <c r="A19" s="8"/>
+      <c r="B19" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="6"/>
-      <c r="B19" s="9" t="s">
-        <v>59</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="6"/>
-      <c r="B20" s="9" t="s">
-        <v>59</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="14.45">
+      <c r="A20" s="8"/>
+      <c r="B20" s="11" t="s">
+        <v>60</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="7"/>
-      <c r="B21" s="10" t="s">
-        <v>59</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="14.45">
+      <c r="A21" s="9"/>
+      <c r="B21" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F21" s="4">
         <v>789167632</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22" s="8" t="s">
+    <row r="22" spans="1:6" ht="14.45">
+      <c r="A22" s="7" t="s">
         <v>74</v>
       </c>
+      <c r="B22" s="10" t="s">
+        <v>75</v>
+      </c>
       <c r="C22" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F22" s="2">
         <v>775810336</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>74</v>
+    <row r="23" spans="1:6" ht="14.45">
+      <c r="A23" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>75</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F23" s="2">
         <v>778525987</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>74</v>
+    <row r="24" spans="1:6" ht="14.45">
+      <c r="A24" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>75</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F24" s="2">
         <v>772104981</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>74</v>
+    <row r="25" spans="1:6" ht="14.45">
+      <c r="A25" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>75</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F25" s="2">
         <v>772107591</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="1:6" ht="14.45">
+      <c r="A26" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>86</v>
+      <c r="B26" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F26" s="2">
         <v>777410048</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>86</v>
+    <row r="27" spans="1:6" ht="14.45">
+      <c r="A27" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>87</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F27" s="2">
         <v>787656877</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>86</v>
+    <row r="28" spans="1:6" ht="14.45">
+      <c r="A28" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>87</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F28" s="2">
         <v>776019823</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>86</v>
+    <row r="29" spans="1:6" ht="14.45">
+      <c r="A29" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>87</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F29" s="2">
         <v>782981141</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>99</v>
+    <row r="30" spans="1:6" ht="14.45">
+      <c r="A30" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>100</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F30" s="2">
         <v>788255458</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>99</v>
+    <row r="31" spans="1:6" ht="14.45">
+      <c r="A31" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>100</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F31" s="2">
         <v>789166919</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>99</v>
+    <row r="32" spans="1:6" ht="14.45">
+      <c r="A32" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>100</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F32" s="2">
         <v>789151415</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>99</v>
+    <row r="33" spans="1:6" ht="14.45">
+      <c r="A33" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>100</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F33" s="2">
         <v>789166998</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>111</v>
+    <row r="34" spans="1:6" ht="14.45">
+      <c r="A34" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F34" s="2">
         <v>781180310</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="6"/>
-      <c r="B35" s="9" t="s">
-        <v>111</v>
+    <row r="35" spans="1:6" ht="14.45">
+      <c r="A35" s="8"/>
+      <c r="B35" s="11" t="s">
+        <v>112</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F35" s="2">
         <v>781180552</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="6"/>
-      <c r="B36" s="9" t="s">
-        <v>111</v>
+    <row r="36" spans="1:6" ht="14.45">
+      <c r="A36" s="8"/>
+      <c r="B36" s="11" t="s">
+        <v>112</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F36" s="2">
         <v>787080588</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="7"/>
-      <c r="B37" s="10" t="s">
-        <v>111</v>
+    <row r="37" spans="1:6" ht="14.45">
+      <c r="A37" s="9"/>
+      <c r="B37" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F37" s="2">
         <v>789150406</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>123</v>
+    <row r="38" spans="1:6" ht="14.45">
+      <c r="A38" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>124</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F38" s="2">
         <v>771545210</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>123</v>
+    <row r="39" spans="1:6" ht="14.45">
+      <c r="A39" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>124</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F39" s="2">
         <v>773958904</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>123</v>
+    <row r="40" spans="1:6" ht="14.45">
+      <c r="A40" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>124</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F40" s="2">
         <v>776950987</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>123</v>
+    <row r="41" spans="1:6">
+      <c r="A41" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>124</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F41" s="2">
         <v>781825193</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" ht="14.45" customHeight="1">
       <c r="A42" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B42" s="8" t="s">
-        <v>135</v>
+      <c r="B42" s="10" t="s">
+        <v>136</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F42" s="2">
         <v>786180521</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" ht="14.45" customHeight="1">
       <c r="A43" s="6"/>
-      <c r="B43" s="9" t="s">
-        <v>135</v>
+      <c r="B43" s="11" t="s">
+        <v>136</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F43" s="2">
         <v>786183517</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" ht="14.45" customHeight="1">
       <c r="A44" s="6"/>
-      <c r="B44" s="9" t="s">
-        <v>135</v>
+      <c r="B44" s="11" t="s">
+        <v>136</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F44" s="2">
         <v>772118585</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="7"/>
-      <c r="B45" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E45" s="2" t="s">
+    <row r="45" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A45" s="6"/>
+      <c r="B45" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D45" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="F45" s="2">
+      <c r="E45" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="F45" s="15">
         <v>787389275</v>
       </c>
     </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="F46" s="14">
+        <v>785249423</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="16"/>
+      <c r="B47" s="17"/>
+      <c r="C47" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="F47" s="14">
+        <v>784720703</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="16"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F48" s="14">
+        <v>787979910</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="16"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="F49" s="14">
+        <v>789514893</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F45"/>
-  <mergeCells count="22">
+  <autoFilter ref="A1:F45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <mergeCells count="23">
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B22:B25"/>
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="B38:B41"/>
-    <mergeCell ref="A42:A45"/>
     <mergeCell ref="B42:B45"/>
     <mergeCell ref="A26:A29"/>
     <mergeCell ref="B26:B29"/>
@@ -1761,18 +1939,6 @@
     <mergeCell ref="B30:B33"/>
     <mergeCell ref="A34:A37"/>
     <mergeCell ref="B34:B37"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="B10:B13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
MAJ fichier Liste VTO.xlsx
</commit_message>
<xml_diff>
--- a/Liste VTO.xlsx
+++ b/Liste VTO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dossier LOUMA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sonatelworkplace-my.sharepoint.com/personal/fall7435_orange-sonatel_com/Documents/Bureau/DOSSIER LOUMAS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="11_62E75E214BEF08387827ABE3F4F2BDEBE23AB00D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDCB5D04-E430-4269-A0E8-20CA2EEAA14D}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{40ED9D43-4F44-4B93-A6D3-4D729016E810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A826E40-2501-45FB-970F-133BFF453CF7}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste VTO" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="162">
   <si>
     <t>DRV</t>
   </si>
@@ -119,9 +119,6 @@
     <t>LO</t>
   </si>
   <si>
-    <t>pvt_smmc2928</t>
-  </si>
-  <si>
     <t>GAMOU</t>
   </si>
   <si>
@@ -203,9 +200,6 @@
     <t>pvt_mbpling0268</t>
   </si>
   <si>
-    <t xml:space="preserve">Fallou </t>
-  </si>
-  <si>
     <t>pvt_mbpling0274</t>
   </si>
   <si>
@@ -353,30 +347,9 @@
     <t>NORD</t>
   </si>
   <si>
-    <t>ALLA  SOW</t>
-  </si>
-  <si>
-    <t>Pvt_tdc590043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABIBOU  </t>
-  </si>
-  <si>
     <t>DIOP</t>
   </si>
   <si>
-    <t>Pvt_tdc590120</t>
-  </si>
-  <si>
-    <t>BILALY</t>
-  </si>
-  <si>
-    <t>BASSOUM</t>
-  </si>
-  <si>
-    <t>Pvt_tdc590016</t>
-  </si>
-  <si>
     <t>PVT FOFANA SORIKE KEDOUGOU (RAVT ZONE KEDOUGOU)</t>
   </si>
   <si>
@@ -452,57 +425,18 @@
     <t>PVT TOUBA BOGO COMMUNICATION (ZONE MBOUR)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gnima </t>
-  </si>
-  <si>
-    <t>Diatta</t>
-  </si>
-  <si>
     <t>pvt_tbogo1367</t>
   </si>
   <si>
-    <t>Rose Mendy</t>
-  </si>
-  <si>
-    <t>Mendy</t>
-  </si>
-  <si>
     <t>pvt_tbogo1124</t>
   </si>
   <si>
-    <t xml:space="preserve">Pauline coumba </t>
-  </si>
-  <si>
-    <t>Faye</t>
-  </si>
-  <si>
     <t>pvt_tbogo1534</t>
   </si>
   <si>
-    <t>Fall</t>
-  </si>
-  <si>
-    <t>pvt_tbogo1719</t>
-  </si>
-  <si>
     <t>IBRAHIMA SENE(SADI ZPPG)</t>
   </si>
   <si>
-    <t xml:space="preserve">KHADIM </t>
-  </si>
-  <si>
-    <t>NIANG</t>
-  </si>
-  <si>
-    <t>Pvt_ibsen0464</t>
-  </si>
-  <si>
-    <t>CHEIKH</t>
-  </si>
-  <si>
-    <t>Pvt_ibsen0440</t>
-  </si>
-  <si>
     <t xml:space="preserve">BOUSSO </t>
   </si>
   <si>
@@ -519,13 +453,85 @@
   </si>
   <si>
     <t>Pvt_ibsen0239</t>
+  </si>
+  <si>
+    <t>pvt_smmc3467</t>
+  </si>
+  <si>
+    <t>Pvt_tdc590313</t>
+  </si>
+  <si>
+    <t>DIAW</t>
+  </si>
+  <si>
+    <t>BASSIROU</t>
+  </si>
+  <si>
+    <t>MATY</t>
+  </si>
+  <si>
+    <t>KA</t>
+  </si>
+  <si>
+    <t>Pvt_tdc590014</t>
+  </si>
+  <si>
+    <t>MMAME KHASS</t>
+  </si>
+  <si>
+    <t>SYLLA</t>
+  </si>
+  <si>
+    <t>Pvt_tdc590021</t>
+  </si>
+  <si>
+    <t>ASSANE</t>
+  </si>
+  <si>
+    <t>pvt_tbogo1864</t>
+  </si>
+  <si>
+    <t>GNIMA</t>
+  </si>
+  <si>
+    <t>DIATTA</t>
+  </si>
+  <si>
+    <t>LOUISE MAME LISSA</t>
+  </si>
+  <si>
+    <t>Pvt_ibsen0551</t>
+  </si>
+  <si>
+    <t>MAREME</t>
+  </si>
+  <si>
+    <t>TOURE</t>
+  </si>
+  <si>
+    <t>Pvt_ibsen0550</t>
+  </si>
+  <si>
+    <t>FALLOU</t>
+  </si>
+  <si>
+    <t>ROSE</t>
+  </si>
+  <si>
+    <t>MENDY</t>
+  </si>
+  <si>
+    <t>FAYE</t>
+  </si>
+  <si>
+    <t>PAULINE COUMBA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -554,7 +560,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -564,6 +570,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -660,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -675,6 +687,13 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -694,15 +713,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -984,16 +998,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="58.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="2" max="2" width="58.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1013,11 +1027,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1033,9 +1047,9 @@
         <v>782989910</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A3" s="8"/>
-      <c r="B3" s="11"/>
+    <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="11"/>
+      <c r="B3" s="14"/>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1049,9 +1063,9 @@
         <v>787095594</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="8"/>
-      <c r="B4" s="11"/>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="11"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1065,9 +1079,9 @@
         <v>781180981</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="9"/>
-      <c r="B5" s="12"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="12"/>
+      <c r="B5" s="15"/>
       <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1081,11 +1095,11 @@
         <v>787095584</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -1097,825 +1111,832 @@
       <c r="E6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="2">
-        <v>786241266</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="14.45">
-      <c r="A7" s="8"/>
-      <c r="B7" s="11" t="s">
+      <c r="F6" s="4">
+        <v>781990323</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="11"/>
+      <c r="B7" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F7" s="4">
+        <v>710019414</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="11"/>
+      <c r="B8" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="2">
-        <v>789160174</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="14.45">
-      <c r="A8" s="8"/>
-      <c r="B8" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="F8" s="2">
         <v>786241255</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.45">
-      <c r="A9" s="9"/>
-      <c r="B9" s="12" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="12"/>
+      <c r="B9" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="4">
+        <v>789160171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="2">
-        <v>775812208</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.45">
-      <c r="A10" s="7" t="s">
+      <c r="B10" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="F10" s="2">
         <v>789166714</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.45">
-      <c r="A11" s="8"/>
-      <c r="B11" s="11" t="s">
-        <v>33</v>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="11"/>
+      <c r="B11" s="14" t="s">
+        <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="3" t="s">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="11"/>
+      <c r="B12" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="14.45">
-      <c r="A12" s="8"/>
-      <c r="B12" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" s="2">
         <v>789166702</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.45">
-      <c r="A13" s="9"/>
-      <c r="B13" s="12" t="s">
-        <v>33</v>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="12"/>
+      <c r="B13" s="15" t="s">
+        <v>32</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="F13" s="2">
         <v>787655205</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="14.45">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="C14" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.45">
-      <c r="A15" s="8"/>
-      <c r="B15" s="11" t="s">
-        <v>47</v>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="11"/>
+      <c r="B15" s="14" t="s">
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="F15" s="2">
         <v>787080726</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="14.45">
-      <c r="A16" s="8"/>
-      <c r="B16" s="11" t="s">
-        <v>47</v>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="11"/>
+      <c r="B16" s="14" t="s">
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>54</v>
+        <v>157</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F16" s="2">
         <v>787081068</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="14.45">
-      <c r="A17" s="9"/>
-      <c r="B17" s="12" t="s">
-        <v>47</v>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="12"/>
+      <c r="B17" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="F17" s="2">
         <v>781590999</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="14.45">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="D18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="F18" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="11"/>
+      <c r="B19" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="D19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="14.45">
-      <c r="A19" s="8"/>
-      <c r="B19" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="F19" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="2" t="s">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="11"/>
+      <c r="B20" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="14.45">
-      <c r="A20" s="8"/>
-      <c r="B20" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="2" t="s">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="12"/>
+      <c r="B21" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="14.45">
-      <c r="A21" s="9"/>
-      <c r="B21" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="F21" s="16">
+        <v>789167632</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="B22" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="F21" s="4">
-        <v>789167632</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="14.45">
-      <c r="A22" s="7" t="s">
+      <c r="C22" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="D22" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="F22" s="2">
         <v>775810336</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="14.45">
-      <c r="A23" s="8" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="F23" s="2">
         <v>778525987</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="14.45">
-      <c r="A24" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>75</v>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>73</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F24" s="2">
         <v>772104981</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="14.45">
-      <c r="A25" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>75</v>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F25" s="2">
         <v>772107591</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="14.45">
-      <c r="A26" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" s="10" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="F26" s="2">
         <v>777410048</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="14.45">
-      <c r="A27" s="8" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="F27" s="2">
         <v>787656877</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="14.45">
-      <c r="A28" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>87</v>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>85</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="F28" s="2">
         <v>776019823</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="14.45">
-      <c r="A29" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>87</v>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="F29" s="2">
         <v>782981141</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="14.45">
-      <c r="A30" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="10" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="F30" s="2">
         <v>788255458</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="14.45">
-      <c r="A31" s="8" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F31" s="4">
+        <v>789157751</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32" s="4">
+        <v>789166902</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="4">
+        <v>710015134</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="B31" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="D34" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F31" s="2">
-        <v>789166919</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="14.45">
-      <c r="A32" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="E34" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F32" s="2">
-        <v>789151415</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="14.45">
-      <c r="A33" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F33" s="2">
-        <v>789166998</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="14.45">
-      <c r="A34" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="F34" s="2">
         <v>781180310</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="14.45">
-      <c r="A35" s="8"/>
-      <c r="B35" s="11" t="s">
-        <v>112</v>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="11"/>
+      <c r="B35" s="14" t="s">
+        <v>103</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="F35" s="2">
         <v>781180552</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="14.45">
-      <c r="A36" s="8"/>
-      <c r="B36" s="11" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="11"/>
+      <c r="B36" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="F36" s="2">
         <v>787080588</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="14.45">
-      <c r="A37" s="9"/>
-      <c r="B37" s="12" t="s">
-        <v>112</v>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="12"/>
+      <c r="B37" s="15" t="s">
+        <v>103</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="F37" s="2">
         <v>789150406</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="14.45">
-      <c r="A38" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>124</v>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="F38" s="2">
         <v>771545210</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="14.45">
-      <c r="A39" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>124</v>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>115</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="F39" s="2">
         <v>773958904</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="14.45">
-      <c r="A40" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>124</v>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>115</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="F40" s="2">
         <v>776950987</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B41" s="12" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>133</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="F41" s="2">
         <v>781825193</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="14.45" customHeight="1">
+    <row r="42" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B42" s="10" t="s">
-        <v>136</v>
+      <c r="B42" s="13" t="s">
+        <v>127</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="F42" s="2">
         <v>786180521</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="14.45" customHeight="1">
+    <row r="43" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6"/>
-      <c r="B43" s="11" t="s">
-        <v>136</v>
+      <c r="B43" s="14" t="s">
+        <v>127</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="F43" s="2">
         <v>786183517</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="14.45" customHeight="1">
+    <row r="44" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6"/>
-      <c r="B44" s="11" t="s">
-        <v>136</v>
+      <c r="B44" s="14" t="s">
+        <v>127</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="F44" s="2">
         <v>772118585</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="14.45" customHeight="1">
+    <row r="45" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6"/>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="E45" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="F45" s="17">
+        <v>789157530</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="D46" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E46" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="F46" s="18">
+        <v>789217447</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="8"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="E47" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="F47" s="18">
+        <v>783059147</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="8"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F48" s="7">
+        <v>787979910</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="8"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="C45" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="D45" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="E45" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="F45" s="15">
-        <v>787389275</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
-      <c r="A46" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="B46" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="C46" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="D46" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E46" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="F46" s="14">
-        <v>785249423</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
-      <c r="A47" s="16"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="D47" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="F47" s="14">
-        <v>784720703</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
-      <c r="A48" s="16"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="D48" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F48" s="14">
-        <v>787979910</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49" s="16"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="F49" s="14">
+      <c r="E49" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F49" s="7">
         <v>789514893</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="23">
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B34:B37"/>
     <mergeCell ref="A46:A49"/>
     <mergeCell ref="B46:B49"/>
     <mergeCell ref="A2:A5"/>
@@ -1932,13 +1953,6 @@
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B34:B37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>